<commit_message>
feat: integrar MLflow al entrenamiento con Model Registry y alias champion
</commit_message>
<xml_diff>
--- a/Plan de Trabajo.xlsx
+++ b/Plan de Trabajo.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mgbov\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/05859b30bfd608ff/Documentos/Especializacion en IA -CEIA/Operaciones de aprendizaje automatico 1/TP/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE05D9A3-CA76-42AE-B10E-D9E6D2351CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="4" documentId="13_ncr:1_{CE05D9A3-CA76-42AE-B10E-D9E6D2351CFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{136F827D-2FF4-4683-B6C8-A57D171F911F}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{3A4D3322-599B-4989-A4E8-14F3622FE1E5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3A4D3322-599B-4989-A4E8-14F3622FE1E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="46">
   <si>
     <t>Tarea</t>
   </si>
@@ -177,9 +177,6 @@
   </si>
   <si>
     <t>0.5 h por persona</t>
-  </si>
-  <si>
-    <t>Mati</t>
   </si>
 </sst>
 </file>
@@ -643,18 +640,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{35F24F3D-4CD6-4F15-AB9D-F0DAA372635A}">
   <dimension ref="A1:G13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="4.54296875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="96.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.6328125" customWidth="1"/>
+    <col min="1" max="1" width="4.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="96.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>10</v>
       </c>
@@ -677,7 +674,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2">
         <v>0</v>
       </c>
@@ -698,7 +695,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
         <v>0</v>
       </c>
@@ -719,7 +716,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2">
         <v>0</v>
       </c>
@@ -740,7 +737,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>22</v>
       </c>
@@ -763,7 +760,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>22</v>
       </c>
@@ -783,10 +780,10 @@
         <v>24</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>22</v>
       </c>
@@ -806,10 +803,10 @@
         <v>24</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>32</v>
       </c>
@@ -828,7 +825,7 @@
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>32</v>
       </c>
@@ -847,7 +844,7 @@
       <c r="F9" s="1"/>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>32</v>
       </c>
@@ -866,7 +863,7 @@
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>41</v>
       </c>
@@ -885,7 +882,7 @@
       <c r="F11" s="6"/>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>41</v>
       </c>
@@ -904,7 +901,7 @@
       <c r="F12" s="6"/>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>41</v>
       </c>

</xml_diff>